<commit_message>
Expand professor coverage across Finnish universities
</commit_message>
<xml_diff>
--- a/excel/finland_universities_master.xlsx
+++ b/excel/finland_universities_master.xlsx
@@ -3671,7 +3671,7 @@
 
 <file path=xl\worksheets\sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:O9"/>
+  <dimension ref="A1:O24"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -4367,6 +4367,1161 @@
         </is>
       </c>
     </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT University</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering Science</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Heikki Kalviainen</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computer vision; Pattern recognition; Machine learning; AI engineering</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT official profile</t>
+        </is>
+      </c>
+      <c r="K10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lut.fi/en/profiles/heikki-kalviainen</t>
+        </is>
+      </c>
+      <c r="M10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N10" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT official profile was used for role and research focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT University</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering Science</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Lasse Lensu</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computer vision; Pattern recognition; Image analysis; Machine learning</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT official profile</t>
+        </is>
+      </c>
+      <c r="K11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lut.fi/en/profiles/lasse-lensu</t>
+        </is>
+      </c>
+      <c r="M11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N11" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT official profile was used for role and research focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT University</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Engineering Science</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Zhisong Liu</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Associate Professor</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Industrial AI; Machine learning; Computer vision; Autonomous systems</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">13235</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">48</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">LUT official profile</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.lut.fi/en/profiles/zhisong-liu</t>
+        </is>
+      </c>
+      <c r="M12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N12" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O12" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official LUT profile states 13235 citations and h-index 48.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Eastern Finland</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Computing</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Pauli Miettinen</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Data mining; Machine learning; Discrete optimization; Pattern discovery</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UEF official profile</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.uef.fi/en/person/pauli.miettinen</t>
+        </is>
+      </c>
+      <c r="M13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N13" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O13" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UEF official profile used for role and research fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Eastern Finland</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Computing</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Markku Tukiainen</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Human-computer interaction; Learning technologies; Computer science education</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UEF official profile</t>
+        </is>
+      </c>
+      <c r="K14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.uef.fi/en/person/markku.tukiainen</t>
+        </is>
+      </c>
+      <c r="M14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N14" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UEF official profile used for role and research fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Eastern Finland</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Computing</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ville Hautamaki</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Speech processing; Speaker recognition; Biometrics; Audio analysis</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UEF official profile</t>
+        </is>
+      </c>
+      <c r="K15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.uef.fi/en/person/ville.hautamaki</t>
+        </is>
+      </c>
+      <c r="M15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N15" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">UEF official profile used for role and research fields.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Jyvaskyla</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faculty of Information Technology</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Michael Emmerich</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Multi-objective optimization; Bayesian optimization; Data science; Simulation</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JYU official profile</t>
+        </is>
+      </c>
+      <c r="K16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.jyu.fi/en/people/michael-emmerich</t>
+        </is>
+      </c>
+      <c r="M16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N16" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O16" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JYU official profile used for title and research topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Jyvaskyla</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Faculty of Information Technology</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Vagan Terziyan</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Artificial intelligence; Semantic web; Knowledge engineering; Trust systems</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JYU official profile</t>
+        </is>
+      </c>
+      <c r="K17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.jyu.fi/en/people/vagan-terziyan</t>
+        </is>
+      </c>
+      <c r="M17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N17" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O17" t="inlineStr">
+        <is>
+          <t xml:space="preserve">JYU official profile used for title and research topics.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Vaasa</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Technology and Innovations</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Tero Vartiainen</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Information systems; Digital transformation; Human-computer interaction; Organizational communication</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Vaasa official profile</t>
+        </is>
+      </c>
+      <c r="K18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.uwasa.fi/en/person/tero-vartiainen</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N18" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Vaasa official profile used for title and research description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Vaasa</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">School of Management</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Harri Jalonen</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Knowledge management; Artificial intelligence in organizations; Social robotics; Futures studies</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Vaasa official profile</t>
+        </is>
+      </c>
+      <c r="K19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.uwasa.fi/en/person/harri-jalonen</t>
+        </is>
+      </c>
+      <c r="M19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N19" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">University of Vaasa official profile used for title and research description.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken School of Economics</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Management and Organisation</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Denise Salin</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Management and organisation; Workplace bullying; Leadership; Gender and diversity</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4296</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">31</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken official profile</t>
+        </is>
+      </c>
+      <c r="K20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.hanken.fi/en/person/denise-salin</t>
+        </is>
+      </c>
+      <c r="M20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N20" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Hanken profile states citation and h-index figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken School of Economics</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Marketing</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Kaj Storbacka</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Markets and strategy; Sales management; Business model innovation; Customer relationships</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken official profile</t>
+        </is>
+      </c>
+      <c r="K21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.hanken.fi/en/person/kaj-storbacka</t>
+        </is>
+      </c>
+      <c r="M21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N21" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken official profile used for title and research focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken School of Economics</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Department of Economics</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Joacim Tag</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Assistant Professor</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Economics; Applied econometrics; Productivity; Labor markets</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">750</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">11</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Hanken official profile</t>
+        </is>
+      </c>
+      <c r="K22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.hanken.fi/en/person/joacim-tag</t>
+        </is>
+      </c>
+      <c r="M22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N22" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Official Hanken profile states citation and h-index figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abo Akademi University</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computer Science</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Ivan Porres</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Software engineering; Distributed systems; Formal methods; Process modeling</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abo Akademi official profile</t>
+        </is>
+      </c>
+      <c r="K23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.abo.fi/en/people/ivan-porres/</t>
+        </is>
+      </c>
+      <c r="M23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N23" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abo Akademi official profile used for title and research focus.</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abo Akademi University</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Computer Science</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Johan Lilius</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Professor</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Embedded systems; Dependable systems; Software engineering; Computer architecture</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abo Akademi official profile</t>
+        </is>
+      </c>
+      <c r="K24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2026-03-14</t>
+        </is>
+      </c>
+      <c r="L24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">https://www.abo.fi/en/people/johan-lilius/</t>
+        </is>
+      </c>
+      <c r="M24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="N24" t="inlineStr">
+        <is>
+          <t xml:space="preserve"/>
+        </is>
+      </c>
+      <c r="O24" t="inlineStr">
+        <is>
+          <t xml:space="preserve">Abo Akademi official profile used for title and research focus.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>